<commit_message>
feat: sample_tracker creates and is ingested properly by main.py
</commit_message>
<xml_diff>
--- a/data/sample_tracker.xlsx
+++ b/data/sample_tracker.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -47,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,10 +494,8 @@
           <t>2026-102626</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>10/25/2026</t>
-        </is>
+      <c r="D2" s="1" t="n">
+        <v>46320</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -547,10 +549,8 @@
           <t>ARC-2026-FDE94</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
+      <c r="D3" s="1" t="n">
+        <v>46310</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -604,10 +604,8 @@
           <t>2026-KC-11840</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
+      <c r="D4" s="1" t="n">
+        <v>46319</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -661,10 +659,8 @@
           <t>REQ-1001</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
+      <c r="D5" s="1" t="n">
+        <v>46310</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -716,10 +712,8 @@
           <t>FIN-204</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
+      <c r="D6" s="1" t="n">
+        <v>46296</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -767,10 +761,8 @@
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
+      <c r="D7" s="1" t="n">
+        <v>46285</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
@@ -818,10 +810,8 @@
           <t>PT-8890</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
+      <c r="D8" s="1" t="n">
+        <v>46315</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -873,10 +863,8 @@
           <t>LOG-312</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
+      <c r="D9" s="1" t="n">
+        <v>46305</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -995,10 +983,8 @@
           <t>EH-9901</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
+      <c r="D2" s="1" t="n">
+        <v>46249</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1050,10 +1036,8 @@
           <t>SMS-440</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
+      <c r="D3" s="1" t="n">
+        <v>46213</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>